<commit_message>
Slide 2: June blended table carried forward with July column from client funnel file
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
+++ b/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1168,8 +1168,96 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Blended submitted applications (client dashboard)</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>684</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>653</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>-5%</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Blended approved (client dashboard)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>-14%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Blended funded (client dashboard)</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>-34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Blended traded (client dashboard)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>-34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>June figures per the June 2026 review. Bing’s July month splits dark (Jul 1–10), legacy (Jul 11–22, $5,883, 0 apps), rebuilt (Jul 22–31, $4,742, 20 apps).</t>
         </is>

</xml_diff>

<commit_message>
Adversarial review rulings: rebuild framing, Meta policy line, mix-shift decomposition; bidding exclusion re-verified live
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
+++ b/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
@@ -844,7 +844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1171,93 +1171,115 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Blended submitted applications (client dashboard)</t>
+          <t>Four continuing channels spend (excl. new Native/DOOH lines)</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>684</t>
+          <t>$120,393</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>$95,401</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>-5%</t>
+          <t>-21%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Blended approved (client dashboard)</t>
+          <t>Blended submitted applications (client dashboard)</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>684</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>653</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>-14%</t>
+          <t>-5%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Blended funded (client dashboard)</t>
+          <t>Blended approved (client dashboard)</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>180</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>-34%</t>
+          <t>-14%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>Blended funded (client dashboard)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>-34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
           <t>Blended traded (client dashboard)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>-34%</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>June figures per the June 2026 review. Bing’s July month splits dark (Jul 1–10), legacy (Jul 11–22, $5,883, 0 apps), rebuilt (Jul 22–31, $4,742, 20 apps).</t>
         </is>

</xml_diff>

<commit_message>
DOOH slides added from Perion consolidado, June DOOH report format; deck now 16 slides
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
+++ b/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,6 +65,12 @@
       <i val="1"/>
       <color rgb="005A6072"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Georgia"/>
+      <b val="1"/>
+      <color rgb="001E2761"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Georgia"/>
@@ -122,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,6 +158,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -517,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -830,6 +837,143 @@
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Spend per the client budget tracker. Native combines Quantcast’s native placement and Azerion’s native inventory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>DOOH delivery (July, opportunities to see)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Spend ($)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Impressions</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Est. reach (freq 1.8)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Ad plays</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>$15,724</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>825,383</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>458,546</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>$6,040</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>314,817</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>174,898</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Monterrey</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>$5,101</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>265,905</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>147,725</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>$26,865</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>1,406,105</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>781,169</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>126,121</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>DOOH delivery from the vendor consolidado; spend per the client budget tracker. Reach modeled at 1.8 average frequency, the June report convention.</t>
         </is>
       </c>
     </row>
@@ -854,7 +998,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>GGMI — July vs June 2026</t>
         </is>

</xml_diff>

<commit_message>
Permanent reporting rule: per-channel partner signals, combined metric retired, portfolio decisions table
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
+++ b/reports/forex/ggmi/2026-07/output/GGMI-July-2026-Performance-Report.xlsx
@@ -668,12 +668,12 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>41 *</t>
+          <t>41</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>$914.85 *</t>
+          <t>$914.85</t>
         </is>
       </c>
     </row>
@@ -808,33 +808,26 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>* Azerion applications are vendor-reported; Bing applications are SA360-reported (offline-imported into Bing; SA360 is the conversion source of record).</t>
+          <t>Channel results reflect each platform or partner’s reporting methodology and should be interpreted independently.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Conversions come from different systems per channel and are never summed across channels.</t>
+          <t>Cross-channel totals and blended acquisition costs are not used because attribution systems are not directly comparable.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Combined Bing + Azerion view (the one sanctioned pairing): 61 submitted applications at $789.08 (June: 92 at $660.00).</t>
+          <t>Meta clicks are link clicks, the June deck definition. Meta reports on spend and delivery this month.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>Meta clicks are link clicks, the June deck definition. Meta reports on spend and delivery this month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Spend per the client budget tracker. Native combines Quantcast’s native placement and Azerion’s native inventory.</t>
         </is>
@@ -1117,7 +1110,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Azerion apps (vendor-reported)</t>
+          <t>Azerion apps (partner-attributed)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1161,262 +1154,240 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Combined Bing + Azerion apps</t>
+          <t>Quantcast partner-attributed results</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>-31</t>
+          <t>+4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Combined cost per app</t>
+          <t>Quantcast viewability</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>$660.00</t>
+          <t>51.3%</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>$789.08</t>
+          <t>54.45%</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>+19.6%</t>
+          <t>+3.15pp</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Quantcast viewability</t>
+          <t>Azerion viewability (display)</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>51.3%</t>
+          <t>68.5%</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>54.45%</t>
+          <t>82.47%</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>+3.15pp</t>
+          <t>+13.97pp</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Azerion viewability (display)</t>
+          <t>Meta link clicks</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>68.5%</t>
+          <t>407,136</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>82.47%</t>
+          <t>74,489</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>+13.97pp</t>
+          <t>-81.7%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Meta link clicks</t>
+          <t>Mexico sessions (GA4)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>407,136</t>
+          <t>9,236</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>74,489</t>
+          <t>7,310</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>-81.7%</t>
+          <t>-20.9%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Mexico sessions (GA4)</t>
+          <t>Unique visitors, Mexico (GA4)</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>9,236</t>
+          <t>5,838</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>7,310</t>
+          <t>3,981</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>-20.9%</t>
+          <t>-31.8%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Unique visitors, Mexico (GA4)</t>
+          <t>Four continuing channels spend (excl. new Native/DOOH lines)</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>5,838</t>
+          <t>$120,393</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>3,981</t>
+          <t>$95,401</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>-31.8%</t>
+          <t>-21%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Four continuing channels spend (excl. new Native/DOOH lines)</t>
+          <t>Blended submitted applications (client dashboard)</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>$120,393</t>
+          <t>684</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>$95,401</t>
+          <t>653</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>-21%</t>
+          <t>-5%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Blended submitted applications (client dashboard)</t>
+          <t>Blended approved (client dashboard)</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>684</t>
+          <t>209</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>653</t>
+          <t>180</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>-5%</t>
+          <t>-14%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Blended approved (client dashboard)</t>
+          <t>Blended funded (client dashboard)</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>32</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>21</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>-14%</t>
+          <t>-34%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Blended funded (client dashboard)</t>
+          <t>Blended traded (client dashboard)</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>29</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>-34%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>Blended traded (client dashboard)</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>-34%</t>
         </is>

</xml_diff>